<commit_message>
feat: Ajoute les ennemis, les collisions, le score et le Game Over
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_LauppiRyan.xlsx
+++ b/Journal-de-Travail_LauppiRyan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\I320\Projet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9B029AE-AF83-4A30-B6BB-BF5EE67AC35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C445D21-D667-4EEC-825C-2E7A71B2E654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -148,16 +148,34 @@
     <t>J'ai essayé de me connecter a GitHub sans succès par ce que github est moisi</t>
   </si>
   <si>
-    <t>Impossible de recevoir le code par email et d'activer l'A2F</t>
-  </si>
-  <si>
     <t>Je cherchais des idées sur quel jeu j'allais faire</t>
   </si>
   <si>
     <t>J'ai changé de Winform à MonoGames</t>
   </si>
   <si>
-    <t>J'ai commencé  prendre en main MonoGames et j'ai codé le déplacement et les limites</t>
+    <t>J'ai implémenter le tire du projectile dans mon jeu</t>
+  </si>
+  <si>
+    <t>J'ai implémenter les ennemis, leurs déplacement et la collision entre les projectiles et ennemis et la collision entres les ennemis et le joueur</t>
+  </si>
+  <si>
+    <t>Impossible de recevoir le code par email et d'activer l'A2F (qui est obligatoire)</t>
+  </si>
+  <si>
+    <t>J'ai essayé de comprendre ce qu'était le bout de code qui nous a été donné  mais je ne l'ai pas trouvé tres utile</t>
+  </si>
+  <si>
+    <t>J'ai commencé a coder sur Winform mais je comprenais pas grand-chose comme c'était nouveau</t>
+  </si>
+  <si>
+    <t>J'ai crée le repo et le projet sur Github avec la liste des taches</t>
+  </si>
+  <si>
+    <t>J'ai commencé  prendre en main MonoGames et j'ai codé le déplacement du joueur et les limites</t>
+  </si>
+  <si>
+    <t>J'ai créer le rapport et commencé a le completer</t>
   </si>
 </sst>
 </file>
@@ -1165,16 +1183,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>75</c:v>
+                  <c:v>135</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>225</c:v>
+                  <c:v>730</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>105</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2020,16 +2038,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.25</c:v>
+                  <c:v>0.13917525773195877</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.75</c:v>
+                  <c:v>0.75257731958762886</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.10824742268041238</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4264,7 +4282,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>6 heures 0 minutes</v>
+        <v>17 heures 10 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4279,15 +4297,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>240</v>
+        <v>840</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>360</v>
+        <v>1030</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4351,7 +4369,7 @@
       </c>
       <c r="C8" s="31"/>
       <c r="D8" s="32">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E8" s="33" t="s">
         <v>15</v>
@@ -4381,13 +4399,15 @@
       <c r="C9" s="35">
         <v>1</v>
       </c>
-      <c r="D9" s="36"/>
+      <c r="D9" s="36">
+        <v>0</v>
+      </c>
       <c r="E9" s="37"/>
       <c r="F9" s="23" t="s">
         <v>34</v>
       </c>
       <c r="G9" s="40" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="M9" t="s">
         <v>15</v>
@@ -4415,7 +4435,7 @@
         <v>13</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G10" s="39"/>
       <c r="M10" t="s">
@@ -4428,21 +4448,25 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="63" t="str">
+    <row r="11" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="63">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v/>
-      </c>
-      <c r="B11" s="34"/>
-      <c r="C11" s="35"/>
+        <v>36</v>
+      </c>
+      <c r="B11" s="34">
+        <v>45906</v>
+      </c>
+      <c r="C11" s="35">
+        <v>1</v>
+      </c>
       <c r="D11" s="36">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G11" s="40"/>
       <c r="M11" t="s">
@@ -4456,20 +4480,24 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="62" t="str">
+      <c r="A12" s="62">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v/>
-      </c>
-      <c r="B12" s="30"/>
+        <v>36</v>
+      </c>
+      <c r="B12" s="30">
+        <v>45906</v>
+      </c>
       <c r="C12" s="31">
-        <v>3</v>
-      </c>
-      <c r="D12" s="32"/>
+        <v>1</v>
+      </c>
+      <c r="D12" s="32">
+        <v>15</v>
+      </c>
       <c r="E12" s="33" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G12" s="39"/>
       <c r="M12" t="s">
@@ -4483,15 +4511,23 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="63" t="str">
+      <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v/>
-      </c>
-      <c r="B13" s="34"/>
+        <v>36</v>
+      </c>
+      <c r="B13" s="34">
+        <v>45906</v>
+      </c>
       <c r="C13" s="35"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="23"/>
+      <c r="D13" s="36">
+        <v>20</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>36</v>
+      </c>
       <c r="G13" s="40"/>
       <c r="N13">
         <v>6</v>
@@ -4501,15 +4537,23 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="62" t="str">
+      <c r="A14" s="62">
         <f>IF(ISBLANK(B14),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B14))</f>
-        <v/>
-      </c>
-      <c r="B14" s="30"/>
+        <v>36</v>
+      </c>
+      <c r="B14" s="30">
+        <v>45907</v>
+      </c>
       <c r="C14" s="31"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="23"/>
+      <c r="D14" s="32">
+        <v>45</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>42</v>
+      </c>
       <c r="G14" s="39"/>
       <c r="N14">
         <v>7</v>
@@ -4519,15 +4563,25 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="63" t="str">
+      <c r="A15" s="63">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="34"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="23"/>
+        <v>36</v>
+      </c>
+      <c r="B15" s="34">
+        <v>45907</v>
+      </c>
+      <c r="C15" s="35">
+        <v>3</v>
+      </c>
+      <c r="D15" s="36">
+        <v>0</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>43</v>
+      </c>
       <c r="G15" s="40"/>
       <c r="N15">
         <v>8</v>
@@ -4537,45 +4591,75 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="62" t="str">
+      <c r="A16" s="62">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="23"/>
+        <v>38</v>
+      </c>
+      <c r="B16" s="30">
+        <v>45917</v>
+      </c>
+      <c r="C16" s="31">
+        <v>3</v>
+      </c>
+      <c r="D16" s="32">
+        <v>0</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>37</v>
+      </c>
       <c r="G16" s="39"/>
       <c r="O16">
         <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="63" t="str">
+      <c r="A17" s="63">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="34"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="23"/>
+        <v>39</v>
+      </c>
+      <c r="B17" s="34">
+        <v>45924</v>
+      </c>
+      <c r="C17" s="35">
+        <v>4</v>
+      </c>
+      <c r="D17" s="36">
+        <v>0</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>38</v>
+      </c>
       <c r="G17" s="40"/>
       <c r="O17">
         <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="62" t="str">
+      <c r="A18" s="62">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
-        <v/>
-      </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="23"/>
+        <v>39</v>
+      </c>
+      <c r="B18" s="30">
+        <v>45924</v>
+      </c>
+      <c r="C18" s="31">
+        <v>1</v>
+      </c>
+      <c r="D18" s="32">
+        <v>0</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>44</v>
+      </c>
       <c r="G18" s="39"/>
       <c r="O18">
         <v>50</v>
@@ -10886,7 +10970,7 @@
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
@@ -10894,7 +10978,7 @@
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>75</v>
+        <v>135</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10902,11 +10986,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>1 h 15 min</v>
+        <v>2 h 15 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.25</v>
+        <v>0.13917525773195877</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10923,15 +11007,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>180</v>
+        <v>660</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>225</v>
+        <v>730</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10939,11 +11023,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>3 h 45 min</v>
+        <v>12 h 10 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.75</v>
+        <v>0.75257731958762886</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10997,15 +11081,15 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11013,11 +11097,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 00 min</v>
+        <v>1 h 45 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.10824742268041238</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11069,26 +11153,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>180</v>
+        <v>780</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>300</v>
+        <v>970</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>5 h 00 min</v>
+        <v>16 h 10 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>5.5555555555555552E-2</v>
+        <v>0.17962962962962964</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
feat: Ajout des obstacles et correction de bug
Version finale
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_LauppiRyan.xlsx
+++ b/Journal-de-Travail_LauppiRyan.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\I320\Projet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C445D21-D667-4EEC-825C-2E7A71B2E654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09C678DC-18C7-4EFF-8FC9-50ABFD2F7917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="50">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -176,6 +176,21 @@
   </si>
   <si>
     <t>J'ai créer le rapport et commencé a le completer</t>
+  </si>
+  <si>
+    <t>M.Piot à fait l'évaluation des 80%</t>
+  </si>
+  <si>
+    <t>J'ai fait les maquettes des analyses fonctionnelles sur Github</t>
+  </si>
+  <si>
+    <t>J'ai réglé des bugs sur le score la position du pinguin et du Game Over</t>
+  </si>
+  <si>
+    <t>J'ai complété mon JDT</t>
+  </si>
+  <si>
+    <t>J'ai coder les obstacles et fini mon jeu</t>
   </si>
 </sst>
 </file>
@@ -1183,16 +1198,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>135</c:v>
+                  <c:v>155</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>730</c:v>
+                  <c:v>940</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>105</c:v>
+                  <c:v>145</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2038,16 +2053,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.13917525773195877</c:v>
+                  <c:v>0.125</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.75257731958762886</c:v>
+                  <c:v>0.75806451612903225</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.10824742268041238</c:v>
+                  <c:v>0.11693548387096774</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4282,7 +4297,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>17 heures 10 minutes</v>
+        <v>21 heures 40 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4297,15 +4312,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>840</v>
+        <v>1020</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>190</v>
+        <v>280</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1030</v>
+        <v>1300</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4451,10 +4466,10 @@
     <row r="11" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A11" s="63">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B11" s="34">
-        <v>45906</v>
+        <v>45936</v>
       </c>
       <c r="C11" s="35">
         <v>1</v>
@@ -4482,10 +4497,10 @@
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="62">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B12" s="30">
-        <v>45906</v>
+        <v>45936</v>
       </c>
       <c r="C12" s="31">
         <v>1</v>
@@ -4513,10 +4528,10 @@
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B13" s="34">
-        <v>45906</v>
+        <v>45936</v>
       </c>
       <c r="C13" s="35"/>
       <c r="D13" s="36">
@@ -4539,10 +4554,10 @@
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="62">
         <f>IF(ISBLANK(B14),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B14))</f>
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B14" s="30">
-        <v>45907</v>
+        <v>45937</v>
       </c>
       <c r="C14" s="31"/>
       <c r="D14" s="32">
@@ -4565,10 +4580,10 @@
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="63">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B15" s="34">
-        <v>45907</v>
+        <v>45937</v>
       </c>
       <c r="C15" s="35">
         <v>3</v>
@@ -4593,10 +4608,10 @@
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="62">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B16" s="30">
-        <v>45917</v>
+        <v>45954</v>
       </c>
       <c r="C16" s="31">
         <v>3</v>
@@ -4615,13 +4630,13 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A17" s="63">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B17" s="34">
-        <v>45924</v>
+        <v>45954</v>
       </c>
       <c r="C17" s="35">
         <v>4</v>
@@ -4643,10 +4658,10 @@
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="62">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B18" s="30">
-        <v>45924</v>
+        <v>45954</v>
       </c>
       <c r="C18" s="31">
         <v>1</v>
@@ -4666,66 +4681,110 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="63" t="str">
+      <c r="A19" s="63">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
-        <v/>
-      </c>
-      <c r="B19" s="34"/>
+        <v>44</v>
+      </c>
+      <c r="B19" s="34">
+        <v>45957</v>
+      </c>
       <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="23"/>
+      <c r="D19" s="36">
+        <v>30</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>46</v>
+      </c>
       <c r="G19" s="40"/>
       <c r="O19">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="62" t="str">
+      <c r="A20" s="62">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
-        <v/>
-      </c>
-      <c r="B20" s="30"/>
+        <v>44</v>
+      </c>
+      <c r="B20" s="30">
+        <v>45957</v>
+      </c>
       <c r="C20" s="31"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="23"/>
+      <c r="D20" s="32">
+        <v>20</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>45</v>
+      </c>
       <c r="G20" s="39"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="63" t="str">
+      <c r="A21" s="63">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="34"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="23"/>
+        <v>44</v>
+      </c>
+      <c r="B21" s="34">
+        <v>45957</v>
+      </c>
+      <c r="C21" s="35">
+        <v>2</v>
+      </c>
+      <c r="D21" s="36">
+        <v>0</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>47</v>
+      </c>
       <c r="G21" s="40"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="62" t="str">
+      <c r="A22" s="62">
         <f>IF(ISBLANK(B22),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B22))</f>
-        <v/>
-      </c>
-      <c r="B22" s="30"/>
+        <v>44</v>
+      </c>
+      <c r="B22" s="30">
+        <v>45957</v>
+      </c>
       <c r="C22" s="31"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="23"/>
+      <c r="D22" s="32">
+        <v>10</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>48</v>
+      </c>
       <c r="G22" s="39"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="63" t="str">
+      <c r="A23" s="63">
         <f>IF(ISBLANK(B23),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B23))</f>
-        <v/>
-      </c>
-      <c r="B23" s="34"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="23"/>
+        <v>44</v>
+      </c>
+      <c r="B23" s="34">
+        <v>45958</v>
+      </c>
+      <c r="C23" s="35">
+        <v>1</v>
+      </c>
+      <c r="D23" s="36">
+        <v>30</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>49</v>
+      </c>
       <c r="G23" s="40"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -10974,11 +11033,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10986,11 +11045,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>2 h 15 min</v>
+        <v>2 h 35 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.13917525773195877</v>
+        <v>0.125</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11007,15 +11066,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>660</v>
+        <v>840</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>730</v>
+        <v>940</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11023,11 +11082,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>12 h 10 min</v>
+        <v>15 h 40 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.75257731958762886</v>
+        <v>0.75806451612903225</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11085,11 +11144,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>105</v>
+        <v>145</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11097,11 +11156,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>1 h 45 min</v>
+        <v>2 h 25 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.10824742268041238</v>
+        <v>0.11693548387096774</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11153,26 +11212,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>780</v>
+        <v>960</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>190</v>
+        <v>280</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>970</v>
+        <v>1240</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>16 h 10 min</v>
+        <v>20 h 40 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.17962962962962964</v>
+        <v>0.22962962962962963</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>28</v>
@@ -11211,17 +11270,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="a3fb6df6b31548c4fd074caa2ed14580">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3d4691fe5d3e52a7f10faf36b21998c3" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11410,6 +11458,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11420,17 +11479,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48A6C709-6DA4-4E3E-B94B-FDAD41BABC0D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11449,6 +11497,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>